<commit_message>
feat: package from «مبلغ الشريحة» on student import; optional national ID; name + transport number export
- Student import matches «مبلغ الشريحة» to an active package price and assigns it with the
  package's semester dates in one batch (import_assign_packages, migration 0022). No amount or
  an unknown amount: imported without a package (warning). Re-imports keep existing packages.
- Preview shows a count per package and each row's package.
- National number optional again: without it the first password is the transport number;
  an invalid number still rejects the row.
- «تصدير الأسماء وأرقام النقل» on the students and doctors pages (all rows, paged) and on the
  import results; import results now carry the transport number.
- Tests updated and added; demo import file regenerated.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supabase/seed/demo-import.xlsx
+++ b/supabase/seed/demo-import.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:N61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -414,30 +414,33 @@
         <v>الرقم الوطني</v>
       </c>
       <c r="E1" t="str">
+        <v>مبلغ الشريحة</v>
+      </c>
+      <c r="F1" t="str">
         <v>صورة عن البطاقة الجامعية</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>رقم الهاتف المستخدم في الوتس ضمن مجموعة</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>الكلية التابع اليها</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>مكان السكن</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>المنطقة القريبة اليك</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>المنطقة القريبة اليك 2</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>في حال اختيار (أخرى) يرجى كتابة اسم المنقطة القريبة اليك</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>اختر أيام دوامك بالاسبوع</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>متى يبدأ دوامك الاسبوعي</v>
       </c>
     </row>
@@ -455,30 +458,33 @@
         <v>20100330001</v>
       </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>https://drive.google.com/open?id=demo330001</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>0992212102</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>حلب - مشفى النحاس</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>دوار عمر ابوريشة</v>
       </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
       <c r="K2" t="str">
         <v/>
       </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -496,30 +502,33 @@
         <v>20100330002</v>
       </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>https://drive.google.com/open?id=demo330002</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>0997223082</v>
       </c>
-      <c r="G3" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H3" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I3" t="str">
         <v>حلب - دوار الدلة</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>دوار الشرطة</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -537,30 +546,33 @@
         <v>20100330003</v>
       </c>
       <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
         <v>https://drive.google.com/open?id=demo330003</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>0938669467</v>
       </c>
-      <c r="G4" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H4" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I4" t="str">
         <v>حلب - السريان</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>دوار الدلة</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
       <c r="K4" t="str">
         <v/>
       </c>
       <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -578,30 +590,33 @@
         <v>20100330004</v>
       </c>
       <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
         <v>https://drive.google.com/open?id=demo330004</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>0972964049</v>
       </c>
-      <c r="G5" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H5" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I5" t="str">
         <v>حلب - اشارات سوق سيف دولة</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>3000 شقة</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
       <c r="K5" t="str">
         <v/>
       </c>
       <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -619,30 +634,33 @@
         <v>20100330005</v>
       </c>
       <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
         <v>https://drive.google.com/open?id=demo330005</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>0931371815</v>
       </c>
-      <c r="G6" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H6" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I6" t="str">
         <v>حلب - دوار العمارة</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>مشفى النحاس</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
       <c r="K6" t="str">
         <v/>
       </c>
       <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>الساعة ال ١٠ صباحا</v>
       </c>
     </row>
@@ -660,30 +678,33 @@
         <v>20100330006</v>
       </c>
       <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
         <v>https://drive.google.com/open?id=demo330006</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>+963 992 504 947</v>
       </c>
-      <c r="G7" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H7" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I7" t="str">
         <v>حلب - جامع النصر</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>مولات سيف دولة</v>
       </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
       <c r="K7" t="str">
         <v/>
       </c>
       <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M7" t="str">
+      <c r="N7" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -701,30 +722,33 @@
         <v>20100330007</v>
       </c>
       <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
         <v>https://drive.google.com/open?id=demo330007</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>986659663</v>
       </c>
-      <c r="G8" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H8" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I8" t="str">
         <v>حلب - دوار الكرة</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>جوية</v>
       </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
       <c r="K8" t="str">
         <v/>
       </c>
       <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M8" t="str">
+      <c r="N8" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -742,30 +766,33 @@
         <v>20100330008</v>
       </c>
       <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
         <v>https://drive.google.com/open?id=demo330008</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>0983 108 092</v>
       </c>
-      <c r="G9" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H9" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I9" t="str">
         <v>حلب - 3000 شقة</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <v>دوار الشفاء</v>
       </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
       <c r="K9" t="str">
         <v/>
       </c>
       <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M9" t="str">
+      <c r="N9" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -783,30 +810,33 @@
         <v>20100330009</v>
       </c>
       <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
         <v>https://drive.google.com/open?id=demo330009</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>9.86659663E8</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>حلب - ال 1070 شقة</v>
       </c>
-      <c r="I10" t="str">
+      <c r="J10" t="str">
         <v>قرطبة</v>
       </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
       <c r="K10" t="str">
         <v/>
       </c>
       <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M10" t="str">
+      <c r="N10" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -824,30 +854,33 @@
         <v>20100330010</v>
       </c>
       <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
         <v>https://drive.google.com/open?id=demo330010</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>+966565324644</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>حلب - كازية الشياح</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <v>مولات سيف دولة</v>
       </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
       <c r="K11" t="str">
         <v/>
       </c>
       <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M11" t="str">
+      <c r="N11" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -865,30 +898,33 @@
         <v>20100330011</v>
       </c>
       <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
         <v>https://drive.google.com/open?id=demo330011</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>+971501234567</v>
       </c>
-      <c r="G12" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H12" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I12" t="str">
         <v>حلب - دوار الطب العربي</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
         <v>ساحة سعد الله جابري</v>
       </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
       <c r="K12" t="str">
         <v/>
       </c>
       <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M12" t="str">
+      <c r="N12" t="str">
         <v>الساعة ال ١٠ صباحا</v>
       </c>
     </row>
@@ -906,30 +942,33 @@
         <v>20100330012</v>
       </c>
       <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
         <v>https://drive.google.com/open?id=demo330012</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>+905321234567</v>
       </c>
-      <c r="G13" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H13" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I13" t="str">
         <v>حلب - ساحة سعد الله جابري</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
         <v>اشارات الشهباء</v>
       </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
       <c r="K13" t="str">
         <v/>
       </c>
       <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M13" t="str">
+      <c r="N13" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -947,30 +986,33 @@
         <v>20100330013</v>
       </c>
       <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
         <v>https://drive.google.com/open?id=demo330013</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>+96566012345</v>
       </c>
-      <c r="G14" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H14" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I14" t="str">
         <v>حلب - اشارات الشهباء</v>
       </c>
-      <c r="I14" t="str">
+      <c r="J14" t="str">
         <v>اشارات سيرياتيل</v>
       </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
       <c r="K14" t="str">
         <v/>
       </c>
       <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M14" t="str">
+      <c r="N14" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -988,30 +1030,33 @@
         <v>20100330014</v>
       </c>
       <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
         <v>https://drive.google.com/open?id=demo330014</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>+97336001234</v>
       </c>
-      <c r="G15" t="str">
+      <c r="H15" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
         <v>حلب - جامع التوحيد</v>
       </c>
-      <c r="I15" t="str">
+      <c r="J15" t="str">
         <v>دوار الكرة</v>
       </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
       <c r="K15" t="str">
         <v/>
       </c>
       <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M15" t="str">
+      <c r="N15" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1029,30 +1074,33 @@
         <v>20100330015</v>
       </c>
       <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
         <v>https://drive.google.com/open?id=demo330015</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>+4915112345678</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H16" t="str">
         <v>ادارة الاعمال</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>حلب - المهندسين</v>
       </c>
-      <c r="I16" t="str">
+      <c r="J16" t="str">
         <v>محطة الاكسبريس</v>
       </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
       <c r="K16" t="str">
         <v/>
       </c>
       <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M16" t="str">
+      <c r="N16" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -1070,30 +1118,33 @@
         <v>20100330016</v>
       </c>
       <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
         <v>https://drive.google.com/open?id=demo330016</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>0993414856</v>
       </c>
-      <c r="G17" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H17" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I17" t="str">
         <v>حلب - اشارات سوق سيف دولة</v>
       </c>
-      <c r="I17" t="str">
+      <c r="J17" t="str">
         <v>جسر الحج</v>
       </c>
-      <c r="J17" t="str">
-        <v/>
-      </c>
       <c r="K17" t="str">
         <v/>
       </c>
       <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M17" t="str">
+      <c r="N17" t="str">
         <v>الساعة ال ١٠ صباحا</v>
       </c>
     </row>
@@ -1111,30 +1162,33 @@
         <v>20100330017</v>
       </c>
       <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
         <v>https://drive.google.com/open?id=demo330017</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>0988191686</v>
       </c>
-      <c r="G18" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H18" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I18" t="str">
         <v>حلب - مشفى النحاس</v>
       </c>
-      <c r="I18" t="str">
+      <c r="J18" t="str">
         <v>الصنم</v>
       </c>
-      <c r="J18" t="str">
-        <v/>
-      </c>
       <c r="K18" t="str">
         <v/>
       </c>
       <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M18" t="str">
+      <c r="N18" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1152,30 +1206,33 @@
         <v>20100330018</v>
       </c>
       <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
         <v>https://drive.google.com/open?id=demo330018</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>0937269724</v>
       </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H19" t="str">
+      <c r="I19" t="str">
         <v>حلب - دوار الشفاء</v>
       </c>
-      <c r="I19" t="str">
+      <c r="J19" t="str">
         <v>أخرى</v>
       </c>
-      <c r="J19" t="str">
-        <v/>
-      </c>
       <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
         <v>حي الفرقان</v>
       </c>
-      <c r="L19" t="str">
+      <c r="M19" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M19" t="str">
+      <c r="N19" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -1193,30 +1250,33 @@
         <v>20100330019</v>
       </c>
       <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
         <v>https://drive.google.com/open?id=demo330019</v>
       </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
         <v>0944828862</v>
       </c>
-      <c r="G20" t="str">
+      <c r="H20" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
         <v>حلب - جوية</v>
       </c>
-      <c r="I20" t="str">
+      <c r="J20" t="str">
         <v>أخرى</v>
       </c>
-      <c r="J20" t="str">
-        <v/>
-      </c>
       <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
         <v>الشعار</v>
       </c>
-      <c r="L20" t="str">
+      <c r="M20" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M20" t="str">
+      <c r="N20" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -1234,30 +1294,33 @@
         <v>20100330020</v>
       </c>
       <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
         <v>https://drive.google.com/open?id=demo330020</v>
       </c>
-      <c r="F21" t="str">
+      <c r="G21" t="str">
         <v>0982229842</v>
       </c>
-      <c r="G21" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H21" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I21" t="str">
         <v>حلب - اوتستراد الحمدانية</v>
       </c>
-      <c r="I21" t="str">
+      <c r="J21" t="str">
         <v>أخرى</v>
       </c>
-      <c r="J21" t="str">
-        <v/>
-      </c>
       <c r="K21" t="str">
         <v/>
       </c>
       <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M21" t="str">
+      <c r="N21" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1275,30 +1338,33 @@
         <v>20100330021</v>
       </c>
       <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
         <v>https://drive.google.com/open?id=demo330021</v>
       </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
         <v>123009</v>
       </c>
-      <c r="G22" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H22" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I22" t="str">
         <v>حلب - كازية الشياح</v>
       </c>
-      <c r="I22" t="str">
+      <c r="J22" t="str">
         <v>ساحة سعد الله جابري</v>
       </c>
-      <c r="J22" t="str">
-        <v/>
-      </c>
       <c r="K22" t="str">
         <v/>
       </c>
       <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M22" t="str">
+      <c r="N22" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1316,30 +1382,33 @@
         <v>20100330022</v>
       </c>
       <c r="E23" t="str">
+        <v/>
+      </c>
+      <c r="F23" t="str">
         <v>https://drive.google.com/open?id=demo330022</v>
       </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
         <v>099614538e</v>
       </c>
-      <c r="G23" t="str">
+      <c r="H23" t="str">
         <v>ادارة الاعمال</v>
       </c>
-      <c r="H23" t="str">
+      <c r="I23" t="str">
         <v>حلب - دوار الكرة</v>
       </c>
-      <c r="I23" t="str">
+      <c r="J23" t="str">
         <v>صحة</v>
       </c>
-      <c r="J23" t="str">
-        <v/>
-      </c>
       <c r="K23" t="str">
         <v/>
       </c>
       <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M23" t="str">
+      <c r="N23" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1357,30 +1426,33 @@
         <v>20100330023</v>
       </c>
       <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
         <v>https://drive.google.com/open?id=demo330023</v>
       </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
         <v>0942513328</v>
       </c>
-      <c r="G24" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H24" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I24" t="str">
         <v>حلب - اشارات سيرياتيل</v>
       </c>
-      <c r="I24" t="str">
+      <c r="J24" t="str">
         <v>اوتستراد الحمدانية</v>
       </c>
-      <c r="J24" t="str">
+      <c r="K24" t="str">
         <v>جامع النصر</v>
       </c>
-      <c r="K24" t="str">
-        <v/>
-      </c>
       <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M24" t="str">
+      <c r="N24" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -1398,30 +1470,33 @@
         <v>20100330024</v>
       </c>
       <c r="E25" t="str">
+        <v/>
+      </c>
+      <c r="F25" t="str">
         <v>https://drive.google.com/open?id=demo330024</v>
       </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
         <v>0972544841</v>
       </c>
-      <c r="G25" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H25" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I25" t="str">
         <v>حلب - مستودعات الاعظمية</v>
       </c>
-      <c r="I25" t="str">
+      <c r="J25" t="str">
         <v>جوية</v>
       </c>
-      <c r="J25" t="str">
+      <c r="K25" t="str">
         <v>الرجاء</v>
       </c>
-      <c r="K25" t="str">
-        <v/>
-      </c>
       <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M25" t="str">
+      <c r="N25" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1439,30 +1514,33 @@
         <v>20100330025</v>
       </c>
       <c r="E26" t="str">
+        <v/>
+      </c>
+      <c r="F26" t="str">
         <v>https://drive.google.com/open?id=demo330025</v>
       </c>
-      <c r="F26" t="str">
+      <c r="G26" t="str">
         <v>0932339633</v>
       </c>
-      <c r="G26" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H26" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I26" t="str">
         <v>حلب - دوار الشرطة</v>
       </c>
-      <c r="I26" t="str">
+      <c r="J26" t="str">
         <v>الصنم</v>
       </c>
-      <c r="J26" t="str">
+      <c r="K26" t="str">
         <v>أخرى</v>
       </c>
-      <c r="K26" t="str">
+      <c r="L26" t="str">
         <v>الحمدانية الجديدة</v>
       </c>
-      <c r="L26" t="str">
+      <c r="M26" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M26" t="str">
+      <c r="N26" t="str">
         <v>الساعة ال ١٠ صباحا</v>
       </c>
     </row>
@@ -1480,30 +1558,33 @@
         <v>20100330026</v>
       </c>
       <c r="E27" t="str">
+        <v/>
+      </c>
+      <c r="F27" t="str">
         <v>https://drive.google.com/open?id=demo330026</v>
       </c>
-      <c r="F27" t="str">
+      <c r="G27" t="str">
         <v>0936975139</v>
       </c>
-      <c r="G27" t="str">
+      <c r="H27" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H27" t="str">
+      <c r="I27" t="str">
         <v>حلب - دوار الموت</v>
-      </c>
-      <c r="I27" t="str">
-        <v>أخرى</v>
       </c>
       <c r="J27" t="str">
         <v>أخرى</v>
       </c>
       <c r="K27" t="str">
+        <v>أخرى</v>
+      </c>
+      <c r="L27" t="str">
         <v>حلب الجديدة شمالي</v>
       </c>
-      <c r="L27" t="str">
+      <c r="M27" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M27" t="str">
+      <c r="N27" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1521,30 +1602,33 @@
         <v>20100330027</v>
       </c>
       <c r="E28" t="str">
+        <v/>
+      </c>
+      <c r="F28" t="str">
         <v>https://drive.google.com/open?id=demo330027</v>
       </c>
-      <c r="F28" t="str">
+      <c r="G28" t="str">
         <v>0974600003</v>
       </c>
-      <c r="G28" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H28" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I28" t="str">
         <v>حلب - دوار الصخرة</v>
       </c>
-      <c r="I28" t="str">
+      <c r="J28" t="str">
         <v>أخرى</v>
       </c>
-      <c r="J28" t="str">
+      <c r="K28" t="str">
         <v>دوار الشفاء</v>
       </c>
-      <c r="K28" t="str">
+      <c r="L28" t="str">
         <v>حي الفرقان</v>
       </c>
-      <c r="L28" t="str">
+      <c r="M28" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M28" t="str">
+      <c r="N28" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -1562,30 +1646,33 @@
         <v>20100330028</v>
       </c>
       <c r="E29" t="str">
+        <v/>
+      </c>
+      <c r="F29" t="str">
         <v>https://drive.google.com/open?id=demo330028</v>
       </c>
-      <c r="F29" t="str">
+      <c r="G29" t="str">
         <v>0935156674</v>
       </c>
-      <c r="G29" t="str">
+      <c r="H29" t="str">
         <v>كلية الصيدلة</v>
       </c>
-      <c r="H29" t="str">
+      <c r="I29" t="str">
         <v>حلب - صحة</v>
       </c>
-      <c r="I29" t="str">
+      <c r="J29" t="str">
         <v>دوار العمارة</v>
       </c>
-      <c r="J29" t="str">
-        <v/>
-      </c>
       <c r="K29" t="str">
         <v/>
       </c>
       <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M29" t="str">
+      <c r="N29" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -1603,30 +1690,33 @@
         <v>20100330029</v>
       </c>
       <c r="E30" t="str">
+        <v/>
+      </c>
+      <c r="F30" t="str">
         <v>https://drive.google.com/open?id=demo330029</v>
       </c>
-      <c r="F30" t="str">
+      <c r="G30" t="str">
         <v>0943103710</v>
       </c>
-      <c r="G30" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H30" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I30" t="str">
         <v>حلب - مالية</v>
       </c>
-      <c r="I30" t="str">
+      <c r="J30" t="str">
         <v>مالية</v>
       </c>
-      <c r="J30" t="str">
-        <v/>
-      </c>
       <c r="K30" t="str">
         <v/>
       </c>
       <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
         <v>السبت، الأحد،الاثنين</v>
       </c>
-      <c r="M30" t="str">
+      <c r="N30" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1644,30 +1734,33 @@
         <v>20100330030</v>
       </c>
       <c r="E31" t="str">
+        <v/>
+      </c>
+      <c r="F31" t="str">
         <v>https://drive.google.com/open?id=demo330030</v>
       </c>
-      <c r="F31" t="str">
+      <c r="G31" t="str">
         <v>0954362585</v>
       </c>
-      <c r="G31" t="str">
+      <c r="H31" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H31" t="str">
+      <c r="I31" t="str">
         <v>حلب - المهندسين</v>
       </c>
-      <c r="I31" t="str">
+      <c r="J31" t="str">
         <v>قرطبة</v>
       </c>
-      <c r="J31" t="str">
-        <v/>
-      </c>
       <c r="K31" t="str">
         <v/>
       </c>
       <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
         <v>الأحد, الأحد, الإثنين</v>
       </c>
-      <c r="M31" t="str">
+      <c r="N31" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1685,30 +1778,33 @@
         <v>20100330031</v>
       </c>
       <c r="E32" t="str">
+        <v/>
+      </c>
+      <c r="F32" t="str">
         <v>https://drive.google.com/open?id=demo330031</v>
       </c>
-      <c r="F32" t="str">
+      <c r="G32" t="str">
         <v>0931107032</v>
       </c>
-      <c r="G32" t="str">
+      <c r="H32" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H32" t="str">
+      <c r="I32" t="str">
         <v>حلب - جسر الحج</v>
       </c>
-      <c r="I32" t="str">
+      <c r="J32" t="str">
         <v>ساحة جامعة</v>
       </c>
-      <c r="J32" t="str">
-        <v/>
-      </c>
       <c r="K32" t="str">
         <v/>
       </c>
       <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M32" t="str">
+      <c r="N32" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -1726,30 +1822,33 @@
         <v>20100330032</v>
       </c>
       <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
         <v>https://drive.google.com/open?id=demo330032</v>
       </c>
-      <c r="F33" t="str">
+      <c r="G33" t="str">
         <v>0965413534</v>
       </c>
-      <c r="G33" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H33" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I33" t="str">
         <v>حلب - دوار الصخرة</v>
       </c>
-      <c r="I33" t="str">
+      <c r="J33" t="str">
         <v>ال 1070 شقة</v>
       </c>
-      <c r="J33" t="str">
-        <v/>
-      </c>
       <c r="K33" t="str">
         <v/>
       </c>
       <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M33" t="str">
+      <c r="N33" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -1767,30 +1866,33 @@
         <v>20100330033</v>
       </c>
       <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
         <v>https://drive.google.com/open?id=demo330033</v>
       </c>
-      <c r="F34" t="str">
+      <c r="G34" t="str">
         <v>0976821312</v>
       </c>
-      <c r="G34" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H34" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I34" t="str">
         <v>حلب - دوار العمارة</v>
       </c>
-      <c r="I34" t="str">
+      <c r="J34" t="str">
         <v>مشفى النحاس</v>
       </c>
-      <c r="J34" t="str">
-        <v/>
-      </c>
       <c r="K34" t="str">
         <v/>
       </c>
       <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M34" t="str">
+      <c r="N34" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -1808,30 +1910,33 @@
         <v>20100330034</v>
       </c>
       <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
         <v>https://drive.google.com/open?id=demo330034</v>
       </c>
-      <c r="F35" t="str">
+      <c r="G35" t="str">
         <v>0969705834</v>
       </c>
-      <c r="G35" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H35" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I35" t="str">
         <v>حلب - كازية الشياح</v>
       </c>
-      <c r="I35" t="str">
+      <c r="J35" t="str">
         <v>الدوار المائل</v>
       </c>
-      <c r="J35" t="str">
-        <v/>
-      </c>
       <c r="K35" t="str">
         <v/>
       </c>
       <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M35" t="str">
+      <c r="N35" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1849,30 +1954,33 @@
         <v>20100330035</v>
       </c>
       <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
         <v>https://drive.google.com/open?id=demo330035</v>
       </c>
-      <c r="F36" t="str">
+      <c r="G36" t="str">
         <v>0967415111</v>
       </c>
-      <c r="G36" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H36" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I36" t="str">
         <v>حلب - دوار الكرة</v>
       </c>
-      <c r="I36" t="str">
+      <c r="J36" t="str">
         <v>كازية الشياح</v>
       </c>
-      <c r="J36" t="str">
-        <v/>
-      </c>
       <c r="K36" t="str">
         <v/>
       </c>
       <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M36" t="str">
+      <c r="N36" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1890,30 +1998,33 @@
         <v>20100330036</v>
       </c>
       <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
         <v>https://drive.google.com/open?id=demo330036</v>
       </c>
-      <c r="F37" t="str">
+      <c r="G37" t="str">
         <v>0943655117</v>
       </c>
-      <c r="G37" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H37" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I37" t="str">
         <v>حلب - جامع الرحمن</v>
       </c>
-      <c r="I37" t="str">
+      <c r="J37" t="str">
         <v>دوار الشرطة</v>
       </c>
-      <c r="J37" t="str">
-        <v/>
-      </c>
       <c r="K37" t="str">
         <v/>
       </c>
       <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M37" t="str">
+      <c r="N37" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -1931,30 +2042,33 @@
         <v>20100330037</v>
       </c>
       <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
         <v>https://drive.google.com/open?id=demo330037</v>
       </c>
-      <c r="F38" t="str">
+      <c r="G38" t="str">
         <v>0946523333</v>
       </c>
-      <c r="G38" t="str">
+      <c r="H38" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H38" t="str">
+      <c r="I38" t="str">
         <v>حلب - اشارات الشهباء</v>
       </c>
-      <c r="I38" t="str">
+      <c r="J38" t="str">
         <v>ساحة سعد الله جابري</v>
       </c>
-      <c r="J38" t="str">
-        <v/>
-      </c>
       <c r="K38" t="str">
         <v/>
       </c>
       <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M38" t="str">
+      <c r="N38" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -1972,30 +2086,33 @@
         <v>20100330038</v>
       </c>
       <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
         <v>https://drive.google.com/open?id=demo330038</v>
       </c>
-      <c r="F39" t="str">
+      <c r="G39" t="str">
         <v>0973553284</v>
       </c>
-      <c r="G39" t="str">
+      <c r="H39" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H39" t="str">
+      <c r="I39" t="str">
         <v>حلب - 3000 شقة</v>
       </c>
-      <c r="I39" t="str">
+      <c r="J39" t="str">
         <v>دوار الموت</v>
       </c>
-      <c r="J39" t="str">
-        <v/>
-      </c>
       <c r="K39" t="str">
         <v/>
       </c>
       <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M39" t="str">
+      <c r="N39" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2013,30 +2130,33 @@
         <v>20100330039</v>
       </c>
       <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
         <v>https://drive.google.com/open?id=demo330039</v>
       </c>
-      <c r="F40" t="str">
+      <c r="G40" t="str">
         <v>0935179936</v>
       </c>
-      <c r="G40" t="str">
+      <c r="H40" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H40" t="str">
+      <c r="I40" t="str">
         <v>حلب - دوار العمارة</v>
       </c>
-      <c r="I40" t="str">
+      <c r="J40" t="str">
         <v>اشارات سيرياتيل</v>
       </c>
-      <c r="J40" t="str">
-        <v/>
-      </c>
       <c r="K40" t="str">
         <v/>
       </c>
       <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M40" t="str">
+      <c r="N40" t="str">
         <v>الساعة ٩ صباحا</v>
       </c>
     </row>
@@ -2054,30 +2174,33 @@
         <v/>
       </c>
       <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
         <v>https://drive.google.com/open?id=demo330040</v>
       </c>
-      <c r="F41" t="str">
+      <c r="G41" t="str">
         <v>0951522040</v>
       </c>
-      <c r="G41" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H41" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I41" t="str">
         <v>حلب - اشارات سوق سيف دولة</v>
       </c>
-      <c r="I41" t="str">
+      <c r="J41" t="str">
         <v>السريان</v>
       </c>
-      <c r="J41" t="str">
-        <v/>
-      </c>
       <c r="K41" t="str">
         <v/>
       </c>
       <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M41" t="str">
+      <c r="N41" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2095,30 +2218,33 @@
         <v>12ab</v>
       </c>
       <c r="E42" t="str">
+        <v/>
+      </c>
+      <c r="F42" t="str">
         <v>https://drive.google.com/open?id=demo330041</v>
       </c>
-      <c r="F42" t="str">
+      <c r="G42" t="str">
         <v>0959570249</v>
       </c>
-      <c r="G42" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H42" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I42" t="str">
         <v>حلب - الرجاء</v>
       </c>
-      <c r="I42" t="str">
+      <c r="J42" t="str">
         <v>3000 شقة</v>
       </c>
-      <c r="J42" t="str">
-        <v/>
-      </c>
       <c r="K42" t="str">
         <v/>
       </c>
       <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M42" t="str">
+      <c r="N42" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2136,11 +2262,11 @@
         <v>20100330042</v>
       </c>
       <c r="E43" t="str">
+        <v/>
+      </c>
+      <c r="F43" t="str">
         <v>https://drive.google.com/open?id=demo330042</v>
       </c>
-      <c r="F43" t="str">
-        <v/>
-      </c>
       <c r="G43" t="str">
         <v/>
       </c>
@@ -2160,6 +2286,9 @@
         <v/>
       </c>
       <c r="M43" t="str">
+        <v/>
+      </c>
+      <c r="N43" t="str">
         <v/>
       </c>
     </row>
@@ -2177,30 +2306,33 @@
         <v>20100330043</v>
       </c>
       <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
         <v>https://drive.google.com/open?id=demo330043</v>
       </c>
-      <c r="F44" t="str">
+      <c r="G44" t="str">
         <v>0932202608</v>
       </c>
-      <c r="G44" t="str">
+      <c r="H44" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H44" t="str">
+      <c r="I44" t="str">
         <v>حلب - دوار الصخرة</v>
       </c>
-      <c r="I44" t="str">
+      <c r="J44" t="str">
         <v>الصنم</v>
       </c>
-      <c r="J44" t="str">
-        <v/>
-      </c>
       <c r="K44" t="str">
         <v/>
       </c>
       <c r="L44" t="str">
+        <v/>
+      </c>
+      <c r="M44" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M44" t="str">
+      <c r="N44" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -2218,30 +2350,33 @@
         <v>20100330044</v>
       </c>
       <c r="E45" t="str">
+        <v/>
+      </c>
+      <c r="F45" t="str">
         <v>https://drive.google.com/open?id=demo330044</v>
       </c>
-      <c r="F45" t="str">
+      <c r="G45" t="str">
         <v>0938651702</v>
       </c>
-      <c r="G45" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H45" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I45" t="str">
         <v>حلب - دوار عمر ابوريشة</v>
       </c>
-      <c r="I45" t="str">
+      <c r="J45" t="str">
         <v>جامع الرحمن</v>
       </c>
-      <c r="J45" t="str">
-        <v/>
-      </c>
       <c r="K45" t="str">
         <v/>
       </c>
       <c r="L45" t="str">
+        <v/>
+      </c>
+      <c r="M45" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M45" t="str">
+      <c r="N45" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2259,30 +2394,33 @@
         <v>20100330045</v>
       </c>
       <c r="E46" t="str">
+        <v/>
+      </c>
+      <c r="F46" t="str">
         <v>https://drive.google.com/open?id=demo330045</v>
       </c>
-      <c r="F46" t="str">
+      <c r="G46" t="str">
         <v>0958213555</v>
       </c>
-      <c r="G46" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H46" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I46" t="str">
         <v>حلب - اشارات نيوتاون</v>
       </c>
-      <c r="I46" t="str">
+      <c r="J46" t="str">
         <v>مسمكة ابوجاسم</v>
       </c>
-      <c r="J46" t="str">
-        <v/>
-      </c>
       <c r="K46" t="str">
         <v/>
       </c>
       <c r="L46" t="str">
+        <v/>
+      </c>
+      <c r="M46" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M46" t="str">
+      <c r="N46" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2300,30 +2438,33 @@
         <v>20100330046</v>
       </c>
       <c r="E47" t="str">
+        <v/>
+      </c>
+      <c r="F47" t="str">
         <v>https://drive.google.com/open?id=demo330046</v>
       </c>
-      <c r="F47" t="str">
+      <c r="G47" t="str">
         <v>0942785915</v>
       </c>
-      <c r="G47" t="str">
+      <c r="H47" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H47" t="str">
+      <c r="I47" t="str">
         <v>حلب - اشارات الشهباء</v>
       </c>
-      <c r="I47" t="str">
+      <c r="J47" t="str">
         <v>محطة الاكسبريس</v>
       </c>
-      <c r="J47" t="str">
-        <v/>
-      </c>
       <c r="K47" t="str">
         <v/>
       </c>
       <c r="L47" t="str">
+        <v/>
+      </c>
+      <c r="M47" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M47" t="str">
+      <c r="N47" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2341,30 +2482,33 @@
         <v>20100330047</v>
       </c>
       <c r="E48" t="str">
+        <v/>
+      </c>
+      <c r="F48" t="str">
         <v>https://drive.google.com/open?id=demo330047</v>
       </c>
-      <c r="F48" t="str">
+      <c r="G48" t="str">
         <v>0991212233</v>
       </c>
-      <c r="G48" t="str">
+      <c r="H48" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H48" t="str">
+      <c r="I48" t="str">
         <v>حلب - الصنم</v>
       </c>
-      <c r="I48" t="str">
+      <c r="J48" t="str">
         <v>اشارات نيوتاون</v>
       </c>
-      <c r="J48" t="str">
-        <v/>
-      </c>
       <c r="K48" t="str">
         <v/>
       </c>
       <c r="L48" t="str">
+        <v/>
+      </c>
+      <c r="M48" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M48" t="str">
+      <c r="N48" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -2382,30 +2526,33 @@
         <v>20100330048</v>
       </c>
       <c r="E49" t="str">
+        <v/>
+      </c>
+      <c r="F49" t="str">
         <v>https://drive.google.com/open?id=demo330048</v>
       </c>
-      <c r="F49" t="str">
+      <c r="G49" t="str">
         <v>0996643435</v>
       </c>
-      <c r="G49" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H49" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I49" t="str">
         <v>حلب - الرجاء</v>
       </c>
-      <c r="I49" t="str">
+      <c r="J49" t="str">
         <v>دوار الشرطة</v>
       </c>
-      <c r="J49" t="str">
-        <v/>
-      </c>
       <c r="K49" t="str">
         <v/>
       </c>
       <c r="L49" t="str">
+        <v/>
+      </c>
+      <c r="M49" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M49" t="str">
+      <c r="N49" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2423,30 +2570,33 @@
         <v>20100330049</v>
       </c>
       <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
         <v>https://drive.google.com/open?id=demo330049</v>
       </c>
-      <c r="F50" t="str">
+      <c r="G50" t="str">
         <v>0976603292</v>
       </c>
-      <c r="G50" t="str">
+      <c r="H50" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H50" t="str">
+      <c r="I50" t="str">
         <v>حلب - محطة الاكسبريس</v>
       </c>
-      <c r="I50" t="str">
+      <c r="J50" t="str">
         <v>الصنم</v>
       </c>
-      <c r="J50" t="str">
-        <v/>
-      </c>
       <c r="K50" t="str">
         <v/>
       </c>
       <c r="L50" t="str">
+        <v/>
+      </c>
+      <c r="M50" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M50" t="str">
+      <c r="N50" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -2464,30 +2614,33 @@
         <v>20100330050</v>
       </c>
       <c r="E51" t="str">
+        <v/>
+      </c>
+      <c r="F51" t="str">
         <v>https://drive.google.com/open?id=demo330050</v>
       </c>
-      <c r="F51" t="str">
+      <c r="G51" t="str">
         <v>0963385946</v>
       </c>
-      <c r="G51" t="str">
+      <c r="H51" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H51" t="str">
+      <c r="I51" t="str">
         <v>حلب - مستودعات الاعظمية</v>
       </c>
-      <c r="I51" t="str">
+      <c r="J51" t="str">
         <v>دوار الصخرة</v>
       </c>
-      <c r="J51" t="str">
-        <v/>
-      </c>
       <c r="K51" t="str">
         <v/>
       </c>
       <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M51" t="str">
+      <c r="N51" t="str">
         <v>الساعة ال ١٠ صباحا</v>
       </c>
     </row>
@@ -2505,30 +2658,33 @@
         <v>20100330051</v>
       </c>
       <c r="E52" t="str">
+        <v/>
+      </c>
+      <c r="F52" t="str">
         <v>https://drive.google.com/open?id=demo330051</v>
       </c>
-      <c r="F52" t="str">
+      <c r="G52" t="str">
         <v>0963884710</v>
       </c>
-      <c r="G52" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H52" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I52" t="str">
         <v>حلب - اوتستراد الحمدانية</v>
       </c>
-      <c r="I52" t="str">
+      <c r="J52" t="str">
         <v>ساحة جامعة</v>
       </c>
-      <c r="J52" t="str">
-        <v/>
-      </c>
       <c r="K52" t="str">
         <v/>
       </c>
       <c r="L52" t="str">
+        <v/>
+      </c>
+      <c r="M52" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M52" t="str">
+      <c r="N52" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2546,30 +2702,33 @@
         <v>20100330052</v>
       </c>
       <c r="E53" t="str">
+        <v/>
+      </c>
+      <c r="F53" t="str">
         <v>https://drive.google.com/open?id=demo330052</v>
       </c>
-      <c r="F53" t="str">
+      <c r="G53" t="str">
         <v>0953714399</v>
       </c>
-      <c r="G53" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H53" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I53" t="str">
         <v>حلب - السريان</v>
       </c>
-      <c r="I53" t="str">
+      <c r="J53" t="str">
         <v>صحة</v>
       </c>
-      <c r="J53" t="str">
-        <v/>
-      </c>
       <c r="K53" t="str">
         <v/>
       </c>
       <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M53" t="str">
+      <c r="N53" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2587,30 +2746,33 @@
         <v>20100330053</v>
       </c>
       <c r="E54" t="str">
+        <v/>
+      </c>
+      <c r="F54" t="str">
         <v>https://drive.google.com/open?id=demo330053</v>
       </c>
-      <c r="F54" t="str">
+      <c r="G54" t="str">
         <v>0979749799</v>
       </c>
-      <c r="G54" t="str">
+      <c r="H54" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H54" t="str">
+      <c r="I54" t="str">
         <v>حلب - كازية الشياح</v>
       </c>
-      <c r="I54" t="str">
+      <c r="J54" t="str">
         <v>جوية</v>
       </c>
-      <c r="J54" t="str">
-        <v/>
-      </c>
       <c r="K54" t="str">
         <v/>
       </c>
       <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M54" t="str">
+      <c r="N54" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2628,30 +2790,33 @@
         <v>20100330054</v>
       </c>
       <c r="E55" t="str">
+        <v/>
+      </c>
+      <c r="F55" t="str">
         <v>https://drive.google.com/open?id=demo330054</v>
       </c>
-      <c r="F55" t="str">
+      <c r="G55" t="str">
         <v>0944940818</v>
       </c>
-      <c r="G55" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H55" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I55" t="str">
         <v>حلب - مسمكة ابوجاسم</v>
       </c>
-      <c r="I55" t="str">
+      <c r="J55" t="str">
         <v>دوار الطب العربي</v>
       </c>
-      <c r="J55" t="str">
-        <v/>
-      </c>
       <c r="K55" t="str">
         <v/>
       </c>
       <c r="L55" t="str">
+        <v/>
+      </c>
+      <c r="M55" t="str">
         <v>السبت, الأحد, الاثنين</v>
       </c>
-      <c r="M55" t="str">
+      <c r="N55" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2669,30 +2834,33 @@
         <v>20100330055</v>
       </c>
       <c r="E56" t="str">
+        <v/>
+      </c>
+      <c r="F56" t="str">
         <v>https://drive.google.com/open?id=demo330055</v>
       </c>
-      <c r="F56" t="str">
+      <c r="G56" t="str">
         <v>0950292696</v>
       </c>
-      <c r="G56" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H56" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I56" t="str">
         <v>حلب - جامع التوحيد</v>
       </c>
-      <c r="I56" t="str">
+      <c r="J56" t="str">
         <v>الصنم</v>
       </c>
-      <c r="J56" t="str">
-        <v/>
-      </c>
       <c r="K56" t="str">
         <v/>
       </c>
       <c r="L56" t="str">
+        <v/>
+      </c>
+      <c r="M56" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M56" t="str">
+      <c r="N56" t="str">
         <v>الساعة الثانية ظهرا</v>
       </c>
     </row>
@@ -2710,30 +2878,33 @@
         <v>20100330056</v>
       </c>
       <c r="E57" t="str">
+        <v/>
+      </c>
+      <c r="F57" t="str">
         <v>https://drive.google.com/open?id=demo330056</v>
       </c>
-      <c r="F57" t="str">
+      <c r="G57" t="str">
         <v>0979938479</v>
       </c>
-      <c r="G57" t="str">
+      <c r="H57" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H57" t="str">
+      <c r="I57" t="str">
         <v>حلب - دوار الكلمة الاشرفية</v>
       </c>
-      <c r="I57" t="str">
+      <c r="J57" t="str">
         <v>دوار عمر ابوريشة</v>
       </c>
-      <c r="J57" t="str">
-        <v/>
-      </c>
       <c r="K57" t="str">
         <v/>
       </c>
       <c r="L57" t="str">
+        <v/>
+      </c>
+      <c r="M57" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M57" t="str">
+      <c r="N57" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2751,30 +2922,33 @@
         <v>20100330057</v>
       </c>
       <c r="E58" t="str">
+        <v/>
+      </c>
+      <c r="F58" t="str">
         <v>https://drive.google.com/open?id=demo330057</v>
       </c>
-      <c r="F58" t="str">
+      <c r="G58" t="str">
         <v>0961625047</v>
       </c>
-      <c r="G58" t="str">
+      <c r="H58" t="str">
         <v>كلية هندسة معلومات</v>
       </c>
-      <c r="H58" t="str">
+      <c r="I58" t="str">
         <v>حلب - جامع النصر</v>
       </c>
-      <c r="I58" t="str">
+      <c r="J58" t="str">
         <v>جوية</v>
       </c>
-      <c r="J58" t="str">
-        <v/>
-      </c>
       <c r="K58" t="str">
         <v/>
       </c>
       <c r="L58" t="str">
+        <v/>
+      </c>
+      <c r="M58" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء</v>
       </c>
-      <c r="M58" t="str">
+      <c r="N58" t="str">
         <v>الساعة ال ١٢ ظهرا</v>
       </c>
     </row>
@@ -2792,30 +2966,33 @@
         <v>20100330058</v>
       </c>
       <c r="E59" t="str">
+        <v/>
+      </c>
+      <c r="F59" t="str">
         <v>https://drive.google.com/open?id=demo330058</v>
       </c>
-      <c r="F59" t="str">
+      <c r="G59" t="str">
         <v>0937529400</v>
       </c>
-      <c r="G59" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H59" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I59" t="str">
         <v>حلب - مشفى النحاس</v>
       </c>
-      <c r="I59" t="str">
+      <c r="J59" t="str">
         <v>دوار الدلة</v>
       </c>
-      <c r="J59" t="str">
-        <v/>
-      </c>
       <c r="K59" t="str">
         <v/>
       </c>
       <c r="L59" t="str">
+        <v/>
+      </c>
+      <c r="M59" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M59" t="str">
+      <c r="N59" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2833,30 +3010,33 @@
         <v>20100330059</v>
       </c>
       <c r="E60" t="str">
+        <v/>
+      </c>
+      <c r="F60" t="str">
         <v>https://drive.google.com/open?id=demo330059</v>
       </c>
-      <c r="F60" t="str">
+      <c r="G60" t="str">
         <v>0943861309</v>
       </c>
-      <c r="G60" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H60" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I60" t="str">
         <v>حلب - مولات سيف دولة</v>
       </c>
-      <c r="I60" t="str">
+      <c r="J60" t="str">
         <v>المهندسين</v>
       </c>
-      <c r="J60" t="str">
-        <v/>
-      </c>
       <c r="K60" t="str">
         <v/>
       </c>
       <c r="L60" t="str">
+        <v/>
+      </c>
+      <c r="M60" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء, الأربعاء, الخميس</v>
       </c>
-      <c r="M60" t="str">
+      <c r="N60" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
@@ -2874,36 +3054,39 @@
         <v>20100330060</v>
       </c>
       <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
         <v>https://drive.google.com/open?id=demo330060</v>
       </c>
-      <c r="F61" t="str">
+      <c r="G61" t="str">
         <v>0991550798</v>
       </c>
-      <c r="G61" t="str">
-        <v>كلية طب الاسنان</v>
-      </c>
       <c r="H61" t="str">
+        <v>كلية طب الاسنان</v>
+      </c>
+      <c r="I61" t="str">
         <v>حلب - الدوار المائل</v>
       </c>
-      <c r="I61" t="str">
+      <c r="J61" t="str">
         <v>المهندسين</v>
       </c>
-      <c r="J61" t="str">
-        <v/>
-      </c>
       <c r="K61" t="str">
         <v/>
       </c>
       <c r="L61" t="str">
+        <v/>
+      </c>
+      <c r="M61" t="str">
         <v>السبت, الأحد, الاثنين, الثلاثاء</v>
       </c>
-      <c r="M61" t="str">
+      <c r="N61" t="str">
         <v>الساعة ٨ صباحا</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>